<commit_message>
Correct impounded & prohibited calculation formula to P = Z + R and update summary headers
</commit_message>
<xml_diff>
--- a/backend/generated_excel.xlsx
+++ b/backend/generated_excel.xlsx
@@ -368,7 +368,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -430,10 +430,13 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -468,6 +471,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
@@ -668,7 +674,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0"/>
@@ -694,7 +700,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0"/>
@@ -2131,7 +2137,7 @@
               <b val="1"/>
               <color rgb="00000000"/>
             </rPr>
-            <t>RED</t>
+            <t>Red</t>
           </r>
           <r>
             <rPr>
@@ -2286,82 +2292,82 @@
       </c>
       <c r="C5" s="30" t="inlineStr"/>
       <c r="D5" s="4" t="n"/>
-      <c r="E5" s="29" t="inlineStr">
+      <c r="E5" s="31" t="inlineStr">
         <is>
           <t>DANKA STAFF</t>
         </is>
       </c>
       <c r="F5" s="4" t="n"/>
-      <c r="G5" s="29" t="inlineStr">
+      <c r="G5" s="31" t="inlineStr">
         <is>
           <t>POLICE OFFICERS</t>
         </is>
       </c>
       <c r="H5" s="4" t="n"/>
-      <c r="I5" s="29" t="inlineStr">
+      <c r="I5" s="31" t="inlineStr">
         <is>
           <t>TRUCKS WEIGHED</t>
         </is>
       </c>
-      <c r="J5" s="29" t="inlineStr">
+      <c r="J5" s="31" t="inlineStr">
         <is>
           <t>TRUCKS CHARGED</t>
         </is>
       </c>
-      <c r="K5" s="29" t="inlineStr">
+      <c r="K5" s="31" t="inlineStr">
         <is>
           <t>MILEAGE START</t>
         </is>
       </c>
-      <c r="L5" s="29" t="inlineStr">
+      <c r="L5" s="31" t="inlineStr">
         <is>
           <t>MILEAGE END</t>
         </is>
       </c>
-      <c r="M5" s="29" t="inlineStr">
+      <c r="M5" s="31" t="inlineStr">
         <is>
           <t>KMS</t>
         </is>
       </c>
-      <c r="N5" s="29" t="inlineStr">
+      <c r="N5" s="31" t="inlineStr">
         <is>
           <t>MOBILE VEHICLE</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="31" t="n">
+      <c r="B6" s="32" t="n">
         <v>46154</v>
       </c>
       <c r="C6" s="12" t="inlineStr"/>
-      <c r="D6" s="32" t="n"/>
-      <c r="E6" s="33" t="inlineStr">
+      <c r="D6" s="33" t="n"/>
+      <c r="E6" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="G6" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="I6" s="35" t="n">
+      <c r="G6" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="I6" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="J6" s="35" t="n">
+      <c r="J6" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="36" t="n">
+      <c r="K6" s="37" t="n">
         <v>61267</v>
       </c>
-      <c r="L6" s="37" t="n">
+      <c r="L6" s="38" t="n">
         <v>61447</v>
       </c>
-      <c r="M6" s="35">
+      <c r="M6" s="36">
         <f>L6-K6</f>
         <v/>
       </c>
-      <c r="N6" s="35" t="inlineStr">
+      <c r="N6" s="36" t="inlineStr">
         <is>
           <t>KDS042Z</t>
         </is>
@@ -2370,1021 +2376,1021 @@
     <row r="7" ht="15.75" customHeight="1">
       <c r="B7" s="12" t="inlineStr"/>
       <c r="C7" s="12" t="inlineStr"/>
-      <c r="D7" s="32" t="n"/>
-      <c r="E7" s="33" t="inlineStr"/>
-      <c r="G7" s="34" t="inlineStr"/>
-      <c r="J7" s="37" t="n">
+      <c r="D7" s="33" t="n"/>
+      <c r="E7" s="34" t="inlineStr"/>
+      <c r="G7" s="35" t="inlineStr"/>
+      <c r="J7" s="38" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="G8" s="38" t="inlineStr">
+      <c r="G8" s="39" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="J8" s="39">
+      <c r="J8" s="40">
         <f>J7+J6</f>
         <v/>
       </c>
-      <c r="M8" s="39">
+      <c r="M8" s="40">
         <f>M6</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="40" t="inlineStr"/>
-      <c r="C9" s="41" t="n"/>
-      <c r="D9" s="41" t="n"/>
-      <c r="E9" s="42" t="n"/>
-      <c r="F9" s="43" t="inlineStr">
+      <c r="B9" s="41" t="inlineStr"/>
+      <c r="C9" s="42" t="n"/>
+      <c r="D9" s="42" t="n"/>
+      <c r="E9" s="43" t="n"/>
+      <c r="F9" s="44" t="inlineStr">
         <is>
           <t>EXCESS   WEIGHT</t>
         </is>
       </c>
-      <c r="G9" s="42" t="n"/>
-      <c r="H9" s="40" t="inlineStr"/>
-      <c r="I9" s="41" t="n"/>
-      <c r="J9" s="41" t="n"/>
-      <c r="K9" s="41" t="n"/>
-      <c r="L9" s="41" t="n"/>
-      <c r="M9" s="41" t="n"/>
-      <c r="N9" s="42" t="n"/>
+      <c r="G9" s="43" t="n"/>
+      <c r="H9" s="41" t="inlineStr"/>
+      <c r="I9" s="42" t="n"/>
+      <c r="J9" s="42" t="n"/>
+      <c r="K9" s="42" t="n"/>
+      <c r="L9" s="42" t="n"/>
+      <c r="M9" s="42" t="n"/>
+      <c r="N9" s="43" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="B10" s="44" t="inlineStr">
+      <c r="B10" s="45" t="inlineStr">
         <is>
           <t>DATE  WEIGHED</t>
         </is>
       </c>
-      <c r="C10" s="44" t="inlineStr">
+      <c r="C10" s="46" t="inlineStr">
         <is>
           <t>VEHICLE REG</t>
         </is>
       </c>
-      <c r="D10" s="44" t="inlineStr">
+      <c r="D10" s="46" t="inlineStr">
         <is>
           <t>TRANSPORTER</t>
         </is>
       </c>
-      <c r="E10" s="44" t="inlineStr">
+      <c r="E10" s="46" t="inlineStr">
         <is>
           <t>CONFIG.</t>
         </is>
       </c>
-      <c r="F10" s="44" t="inlineStr">
+      <c r="F10" s="46" t="inlineStr">
         <is>
           <t>GVW</t>
         </is>
       </c>
-      <c r="G10" s="44" t="inlineStr">
+      <c r="G10" s="46" t="inlineStr">
         <is>
           <t>AXLE</t>
         </is>
       </c>
-      <c r="H10" s="44" t="inlineStr">
+      <c r="H10" s="46" t="inlineStr">
         <is>
           <t>ORIGIN</t>
         </is>
       </c>
-      <c r="I10" s="44" t="inlineStr">
+      <c r="I10" s="46" t="inlineStr">
         <is>
           <t>DESTIN.</t>
         </is>
       </c>
-      <c r="J10" s="44" t="inlineStr">
+      <c r="J10" s="46" t="inlineStr">
         <is>
           <t>CARGO</t>
         </is>
       </c>
-      <c r="K10" s="44" t="inlineStr">
+      <c r="K10" s="46" t="inlineStr">
         <is>
           <t>COMPUTER OPERATER 
 (DANKA STAFF)</t>
         </is>
       </c>
-      <c r="L10" s="44" t="inlineStr">
+      <c r="L10" s="46" t="inlineStr">
         <is>
           <t>OFFICERS</t>
         </is>
       </c>
-      <c r="M10" s="44" t="inlineStr">
+      <c r="M10" s="46" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
-      <c r="N10" s="44" t="inlineStr">
+      <c r="N10" s="46" t="inlineStr">
         <is>
           <t>ROUTE</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="31" t="n">
+      <c r="B11" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C11" s="34" t="inlineStr">
+      <c r="C11" s="35" t="inlineStr">
         <is>
           <t>KBW781J</t>
         </is>
       </c>
-      <c r="D11" s="34" t="inlineStr">
+      <c r="D11" s="35" t="inlineStr">
         <is>
           <t>OMAR HALEN.</t>
         </is>
       </c>
-      <c r="E11" s="34" t="inlineStr">
+      <c r="E11" s="35" t="inlineStr">
         <is>
           <t>4A</t>
         </is>
       </c>
-      <c r="F11" s="37" t="n">
+      <c r="F11" s="38" t="n">
         <v>7500</v>
       </c>
-      <c r="G11" s="37" t="n">
+      <c r="G11" s="38" t="n">
         <v>7500</v>
       </c>
-      <c r="H11" s="34" t="inlineStr">
+      <c r="H11" s="35" t="inlineStr">
         <is>
           <t>BURUBURU</t>
         </is>
       </c>
-      <c r="I11" s="34" t="inlineStr">
+      <c r="I11" s="35" t="inlineStr">
         <is>
           <t>EASTLIEGH</t>
         </is>
       </c>
-      <c r="J11" s="34" t="inlineStr">
+      <c r="J11" s="35" t="inlineStr">
         <is>
           <t>WATER</t>
         </is>
       </c>
-      <c r="K11" s="33" t="inlineStr">
+      <c r="K11" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L11" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M11" s="33" t="inlineStr">
+      <c r="L11" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M11" s="34" t="inlineStr">
         <is>
           <t>CHARGED</t>
         </is>
       </c>
-      <c r="N11" s="34" t="inlineStr"/>
+      <c r="N11" s="35" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="B12" s="31" t="n">
+      <c r="B12" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C12" s="34" t="inlineStr">
+      <c r="C12" s="35" t="inlineStr">
         <is>
           <t>KCF479D</t>
         </is>
       </c>
-      <c r="D12" s="34" t="inlineStr">
+      <c r="D12" s="35" t="inlineStr">
         <is>
           <t>DUR DUR</t>
         </is>
       </c>
-      <c r="E12" s="34" t="inlineStr">
+      <c r="E12" s="35" t="inlineStr">
         <is>
           <t>4A</t>
         </is>
       </c>
-      <c r="F12" s="37" t="inlineStr">
+      <c r="F12" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G12" s="37" t="inlineStr">
+      <c r="G12" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H12" s="34" t="inlineStr">
+      <c r="H12" s="35" t="inlineStr">
         <is>
           <t>NAKURU</t>
         </is>
       </c>
-      <c r="I12" s="34" t="inlineStr">
+      <c r="I12" s="35" t="inlineStr">
         <is>
           <t>MOMBASA</t>
         </is>
       </c>
-      <c r="J12" s="34" t="inlineStr">
+      <c r="J12" s="35" t="inlineStr">
         <is>
           <t>WATER</t>
         </is>
       </c>
-      <c r="K12" s="33" t="inlineStr">
+      <c r="K12" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L12" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M12" s="33" t="inlineStr">
+      <c r="L12" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M12" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N12" s="34" t="inlineStr"/>
+      <c r="N12" s="35" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="B13" s="31" t="n">
+      <c r="B13" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C13" s="34" t="inlineStr">
+      <c r="C13" s="35" t="inlineStr">
         <is>
           <t>KDV441Q</t>
         </is>
       </c>
-      <c r="D13" s="34" t="inlineStr">
+      <c r="D13" s="35" t="inlineStr">
         <is>
           <t>TAJI.</t>
         </is>
       </c>
-      <c r="E13" s="34" t="inlineStr">
+      <c r="E13" s="35" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="F13" s="37" t="inlineStr">
+      <c r="F13" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G13" s="37" t="inlineStr">
+      <c r="G13" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H13" s="34" t="inlineStr">
+      <c r="H13" s="35" t="inlineStr">
         <is>
           <t>NAKURU</t>
         </is>
       </c>
-      <c r="I13" s="34" t="inlineStr">
+      <c r="I13" s="35" t="inlineStr">
         <is>
           <t>MOMBASA</t>
         </is>
       </c>
-      <c r="J13" s="34" t="inlineStr">
+      <c r="J13" s="35" t="inlineStr">
         <is>
           <t>EMPTY TO OFFLOAD</t>
         </is>
       </c>
-      <c r="K13" s="33" t="inlineStr">
+      <c r="K13" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L13" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M13" s="33" t="inlineStr">
+      <c r="L13" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M13" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N13" s="34" t="inlineStr"/>
+      <c r="N13" s="35" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="B14" s="31" t="n">
+      <c r="B14" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C14" s="34" t="inlineStr">
+      <c r="C14" s="35" t="inlineStr">
         <is>
           <t>KBW781J</t>
         </is>
       </c>
-      <c r="D14" s="34" t="inlineStr">
+      <c r="D14" s="35" t="inlineStr">
         <is>
           <t>OMAR HALEN.</t>
         </is>
       </c>
-      <c r="E14" s="34" t="inlineStr">
+      <c r="E14" s="35" t="inlineStr">
         <is>
           <t>4A</t>
         </is>
       </c>
-      <c r="F14" s="37" t="inlineStr">
+      <c r="F14" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G14" s="37" t="inlineStr">
+      <c r="G14" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H14" s="34" t="inlineStr">
+      <c r="H14" s="35" t="inlineStr">
         <is>
           <t>BURUBURU</t>
         </is>
       </c>
-      <c r="I14" s="34" t="inlineStr">
+      <c r="I14" s="35" t="inlineStr">
         <is>
           <t>EASTLIEGH</t>
         </is>
       </c>
-      <c r="J14" s="34" t="inlineStr">
+      <c r="J14" s="35" t="inlineStr">
         <is>
           <t>WATER</t>
         </is>
       </c>
-      <c r="K14" s="33" t="inlineStr">
+      <c r="K14" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L14" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M14" s="33" t="inlineStr">
+      <c r="L14" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M14" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N14" s="34" t="inlineStr"/>
+      <c r="N14" s="35" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="B15" s="31" t="n">
+      <c r="B15" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C15" s="34" t="inlineStr">
+      <c r="C15" s="35" t="inlineStr">
         <is>
           <t>KDV441Q</t>
         </is>
       </c>
-      <c r="D15" s="34" t="inlineStr">
+      <c r="D15" s="35" t="inlineStr">
         <is>
           <t>TAJI.</t>
         </is>
       </c>
-      <c r="E15" s="34" t="inlineStr">
+      <c r="E15" s="35" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="F15" s="37" t="inlineStr">
+      <c r="F15" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G15" s="37" t="n">
+      <c r="G15" s="38" t="n">
         <v>1250</v>
       </c>
-      <c r="H15" s="34" t="inlineStr">
+      <c r="H15" s="35" t="inlineStr">
         <is>
           <t>NAKURU</t>
         </is>
       </c>
-      <c r="I15" s="34" t="inlineStr">
+      <c r="I15" s="35" t="inlineStr">
         <is>
           <t>MOMBASA</t>
         </is>
       </c>
-      <c r="J15" s="34" t="inlineStr">
+      <c r="J15" s="35" t="inlineStr">
         <is>
           <t>WATER</t>
         </is>
       </c>
-      <c r="K15" s="33" t="inlineStr">
+      <c r="K15" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L15" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M15" s="33" t="inlineStr">
+      <c r="L15" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M15" s="34" t="inlineStr">
         <is>
           <t>WARNED</t>
         </is>
       </c>
-      <c r="N15" s="34" t="inlineStr"/>
+      <c r="N15" s="35" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="B16" s="31" t="n">
+      <c r="B16" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C16" s="34" t="inlineStr">
+      <c r="C16" s="35" t="inlineStr">
         <is>
           <t>KDS874J</t>
         </is>
       </c>
-      <c r="D16" s="34" t="inlineStr">
+      <c r="D16" s="35" t="inlineStr">
         <is>
           <t>ONDA CONCRETE</t>
         </is>
       </c>
-      <c r="E16" s="34" t="inlineStr">
+      <c r="E16" s="35" t="inlineStr">
         <is>
           <t>4*WW|DD||</t>
         </is>
       </c>
-      <c r="F16" s="37" t="inlineStr">
+      <c r="F16" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G16" s="37" t="inlineStr">
+      <c r="G16" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H16" s="34" t="inlineStr">
+      <c r="H16" s="35" t="inlineStr">
         <is>
           <t>KANGEMI</t>
         </is>
       </c>
-      <c r="I16" s="34" t="inlineStr">
+      <c r="I16" s="35" t="inlineStr">
         <is>
           <t>WESTLANDS</t>
         </is>
       </c>
-      <c r="J16" s="34" t="inlineStr">
+      <c r="J16" s="35" t="inlineStr">
         <is>
           <t>CONCRETE MIX</t>
         </is>
       </c>
-      <c r="K16" s="33" t="inlineStr">
+      <c r="K16" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L16" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M16" s="33" t="inlineStr">
+      <c r="L16" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M16" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N16" s="34" t="inlineStr"/>
+      <c r="N16" s="35" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="B17" s="31" t="n">
+      <c r="B17" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C17" s="34" t="inlineStr">
+      <c r="C17" s="35" t="inlineStr">
         <is>
           <t>KDT651M</t>
         </is>
       </c>
-      <c r="D17" s="34" t="inlineStr">
+      <c r="D17" s="35" t="inlineStr">
         <is>
           <t>C MWANIKI</t>
         </is>
       </c>
-      <c r="E17" s="34" t="inlineStr">
+      <c r="E17" s="35" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="F17" s="37" t="inlineStr">
+      <c r="F17" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="37" t="inlineStr">
+      <c r="G17" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H17" s="34" t="inlineStr">
+      <c r="H17" s="35" t="inlineStr">
         <is>
           <t>NAKURU</t>
         </is>
       </c>
-      <c r="I17" s="34" t="inlineStr">
+      <c r="I17" s="35" t="inlineStr">
         <is>
           <t>MOMBASA</t>
         </is>
       </c>
-      <c r="J17" s="34" t="inlineStr">
+      <c r="J17" s="35" t="inlineStr">
         <is>
           <t>FRENCH BEANS</t>
         </is>
       </c>
-      <c r="K17" s="33" t="inlineStr">
+      <c r="K17" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L17" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M17" s="33" t="inlineStr">
+      <c r="L17" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M17" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N17" s="34" t="inlineStr"/>
+      <c r="N17" s="35" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="B18" s="31" t="n">
+      <c r="B18" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C18" s="34" t="inlineStr">
+      <c r="C18" s="35" t="inlineStr">
         <is>
           <t>KDC439L</t>
         </is>
       </c>
-      <c r="D18" s="34" t="inlineStr">
+      <c r="D18" s="35" t="inlineStr">
         <is>
           <t>WAGATUNDU STORES</t>
         </is>
       </c>
-      <c r="E18" s="34" t="inlineStr">
+      <c r="E18" s="35" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="F18" s="37" t="inlineStr">
+      <c r="F18" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G18" s="37" t="inlineStr">
+      <c r="G18" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H18" s="34" t="inlineStr">
+      <c r="H18" s="35" t="inlineStr">
         <is>
           <t>NAKURU</t>
         </is>
       </c>
-      <c r="I18" s="34" t="inlineStr">
+      <c r="I18" s="35" t="inlineStr">
         <is>
           <t>MOMBASA</t>
         </is>
       </c>
-      <c r="J18" s="34" t="inlineStr">
+      <c r="J18" s="35" t="inlineStr">
         <is>
           <t>BEANS</t>
         </is>
       </c>
-      <c r="K18" s="33" t="inlineStr">
+      <c r="K18" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L18" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M18" s="33" t="inlineStr">
+      <c r="L18" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M18" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N18" s="34" t="inlineStr"/>
+      <c r="N18" s="35" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="B19" s="31" t="n">
+      <c r="B19" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C19" s="34" t="inlineStr">
+      <c r="C19" s="35" t="inlineStr">
         <is>
           <t>KDV739N</t>
         </is>
       </c>
-      <c r="D19" s="34" t="inlineStr">
+      <c r="D19" s="35" t="inlineStr">
         <is>
           <t>MWIJABAKAJO</t>
         </is>
       </c>
-      <c r="E19" s="34" t="inlineStr">
+      <c r="E19" s="35" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="F19" s="37" t="inlineStr">
+      <c r="F19" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G19" s="37" t="inlineStr">
+      <c r="G19" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H19" s="34" t="inlineStr">
+      <c r="H19" s="35" t="inlineStr">
         <is>
           <t>KANGEMI</t>
         </is>
       </c>
-      <c r="I19" s="34" t="inlineStr">
+      <c r="I19" s="35" t="inlineStr">
         <is>
           <t>NAIROBI</t>
         </is>
       </c>
-      <c r="J19" s="34" t="inlineStr">
+      <c r="J19" s="35" t="inlineStr">
         <is>
           <t>BLOCKS</t>
         </is>
       </c>
-      <c r="K19" s="33" t="inlineStr">
+      <c r="K19" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L19" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M19" s="33" t="inlineStr">
+      <c r="L19" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M19" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N19" s="34" t="inlineStr"/>
+      <c r="N19" s="35" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="B20" s="31" t="n">
+      <c r="B20" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C20" s="34" t="inlineStr">
+      <c r="C20" s="35" t="inlineStr">
         <is>
           <t>KBJ976Z</t>
         </is>
       </c>
-      <c r="D20" s="34" t="inlineStr">
+      <c r="D20" s="35" t="inlineStr">
         <is>
           <t>BOLD MILLERS</t>
         </is>
       </c>
-      <c r="E20" s="34" t="inlineStr">
+      <c r="E20" s="35" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="F20" s="37" t="inlineStr">
+      <c r="F20" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G20" s="37" t="inlineStr">
+      <c r="G20" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H20" s="34" t="inlineStr">
+      <c r="H20" s="35" t="inlineStr">
         <is>
           <t>NAKURU</t>
         </is>
       </c>
-      <c r="I20" s="34" t="inlineStr">
+      <c r="I20" s="35" t="inlineStr">
         <is>
           <t>MOMBASA</t>
         </is>
       </c>
-      <c r="J20" s="34" t="inlineStr">
+      <c r="J20" s="35" t="inlineStr">
         <is>
           <t>FLOUR</t>
         </is>
       </c>
-      <c r="K20" s="33" t="inlineStr">
+      <c r="K20" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L20" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M20" s="33" t="inlineStr">
+      <c r="L20" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M20" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N20" s="34" t="inlineStr"/>
+      <c r="N20" s="35" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="B21" s="31" t="n">
+      <c r="B21" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C21" s="34" t="inlineStr">
+      <c r="C21" s="35" t="inlineStr">
         <is>
           <t>KDH273N</t>
         </is>
       </c>
-      <c r="D21" s="34" t="inlineStr">
+      <c r="D21" s="35" t="inlineStr">
         <is>
           <t>GUARDIAN PARCEL</t>
         </is>
       </c>
-      <c r="E21" s="34" t="inlineStr">
+      <c r="E21" s="35" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="F21" s="37" t="inlineStr">
+      <c r="F21" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G21" s="37" t="inlineStr">
+      <c r="G21" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H21" s="34" t="inlineStr">
+      <c r="H21" s="35" t="inlineStr">
         <is>
           <t>NAKURU</t>
         </is>
       </c>
-      <c r="I21" s="34" t="inlineStr">
+      <c r="I21" s="35" t="inlineStr">
         <is>
           <t>NAIROBI</t>
         </is>
       </c>
-      <c r="J21" s="34" t="inlineStr">
+      <c r="J21" s="35" t="inlineStr">
         <is>
           <t>PARCELS</t>
         </is>
       </c>
-      <c r="K21" s="33" t="inlineStr">
+      <c r="K21" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L21" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M21" s="33" t="inlineStr">
+      <c r="L21" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M21" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N21" s="34" t="inlineStr"/>
+      <c r="N21" s="35" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="B22" s="31" t="n">
+      <c r="B22" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C22" s="34" t="inlineStr">
+      <c r="C22" s="35" t="inlineStr">
         <is>
           <t>KCS149N</t>
         </is>
       </c>
-      <c r="D22" s="34" t="inlineStr">
+      <c r="D22" s="35" t="inlineStr">
         <is>
           <t>MAMA MILLERS</t>
         </is>
       </c>
-      <c r="E22" s="34" t="inlineStr">
+      <c r="E22" s="35" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="F22" s="37" t="inlineStr">
+      <c r="F22" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G22" s="37" t="inlineStr">
+      <c r="G22" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H22" s="34" t="inlineStr">
+      <c r="H22" s="35" t="inlineStr">
         <is>
           <t>NAKURU</t>
         </is>
       </c>
-      <c r="I22" s="34" t="inlineStr">
+      <c r="I22" s="35" t="inlineStr">
         <is>
           <t>NAIROBI</t>
         </is>
       </c>
-      <c r="J22" s="34" t="inlineStr">
+      <c r="J22" s="35" t="inlineStr">
         <is>
           <t>BREAD</t>
         </is>
       </c>
-      <c r="K22" s="33" t="inlineStr">
+      <c r="K22" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L22" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M22" s="33" t="inlineStr">
+      <c r="L22" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M22" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N22" s="34" t="inlineStr"/>
+      <c r="N22" s="35" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="B23" s="31" t="n">
+      <c r="B23" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C23" s="34" t="inlineStr">
+      <c r="C23" s="35" t="inlineStr">
         <is>
           <t>KDW642Z</t>
         </is>
       </c>
-      <c r="D23" s="34" t="inlineStr">
+      <c r="D23" s="35" t="inlineStr">
         <is>
           <t>KIJU</t>
         </is>
       </c>
-      <c r="E23" s="34" t="inlineStr">
+      <c r="E23" s="35" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="F23" s="37" t="inlineStr">
+      <c r="F23" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G23" s="37" t="n">
+      <c r="G23" s="38" t="n">
         <v>1800</v>
       </c>
-      <c r="H23" s="34" t="inlineStr">
+      <c r="H23" s="35" t="inlineStr">
         <is>
           <t>NAKURU</t>
         </is>
       </c>
-      <c r="I23" s="34" t="inlineStr">
+      <c r="I23" s="35" t="inlineStr">
         <is>
           <t>MOMBASA</t>
         </is>
       </c>
-      <c r="J23" s="34" t="inlineStr">
+      <c r="J23" s="35" t="inlineStr">
         <is>
           <t>POTATOES</t>
         </is>
       </c>
-      <c r="K23" s="33" t="inlineStr">
+      <c r="K23" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L23" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M23" s="33" t="inlineStr">
+      <c r="L23" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M23" s="34" t="inlineStr">
         <is>
           <t>WARNED</t>
         </is>
       </c>
-      <c r="N23" s="34" t="inlineStr"/>
+      <c r="N23" s="35" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="B24" s="31" t="n">
+      <c r="B24" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C24" s="34" t="inlineStr">
+      <c r="C24" s="35" t="inlineStr">
         <is>
           <t>KDL304J</t>
         </is>
       </c>
-      <c r="D24" s="34" t="inlineStr">
+      <c r="D24" s="35" t="inlineStr">
         <is>
           <t>SUSAN OIRO</t>
         </is>
       </c>
-      <c r="E24" s="34" t="inlineStr">
+      <c r="E24" s="35" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="F24" s="37" t="inlineStr">
+      <c r="F24" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G24" s="37" t="inlineStr">
+      <c r="G24" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H24" s="34" t="inlineStr">
+      <c r="H24" s="35" t="inlineStr">
         <is>
           <t>LIMURU</t>
         </is>
       </c>
-      <c r="I24" s="34" t="inlineStr">
+      <c r="I24" s="35" t="inlineStr">
         <is>
           <t>WESTLANDS</t>
         </is>
       </c>
-      <c r="J24" s="34" t="inlineStr">
+      <c r="J24" s="35" t="inlineStr">
         <is>
           <t>MILK</t>
         </is>
       </c>
-      <c r="K24" s="33" t="inlineStr">
+      <c r="K24" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L24" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M24" s="33" t="inlineStr">
+      <c r="L24" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M24" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N24" s="34" t="inlineStr"/>
+      <c r="N24" s="35" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="B25" s="31" t="n">
+      <c r="B25" s="32" t="n">
         <v>46154</v>
       </c>
-      <c r="C25" s="34" t="inlineStr">
+      <c r="C25" s="35" t="inlineStr">
         <is>
           <t>KDV915V</t>
         </is>
       </c>
-      <c r="D25" s="34" t="inlineStr">
+      <c r="D25" s="35" t="inlineStr">
         <is>
           <t>KINGSMIL</t>
         </is>
       </c>
-      <c r="E25" s="34" t="inlineStr">
+      <c r="E25" s="35" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="F25" s="37" t="inlineStr">
+      <c r="F25" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G25" s="37" t="inlineStr">
+      <c r="G25" s="38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H25" s="34" t="inlineStr">
+      <c r="H25" s="35" t="inlineStr">
         <is>
           <t>NAKURU</t>
         </is>
       </c>
-      <c r="I25" s="34" t="inlineStr">
+      <c r="I25" s="35" t="inlineStr">
         <is>
           <t>MOMBASA</t>
         </is>
       </c>
-      <c r="J25" s="34" t="inlineStr">
+      <c r="J25" s="35" t="inlineStr">
         <is>
           <t>BREAD</t>
         </is>
       </c>
-      <c r="K25" s="33" t="inlineStr">
+      <c r="K25" s="34" t="inlineStr">
         <is>
           <t>DM DUNCAN ODHIAMBO/DM ELIZABETH CHARI/DRIVER SILAS MWANGI</t>
         </is>
       </c>
-      <c r="L25" s="34" t="inlineStr">
-        <is>
-          <t>CPL EMASON SAUTET / PC (W) JANE EKADELI</t>
-        </is>
-      </c>
-      <c r="M25" s="33" t="inlineStr">
+      <c r="L25" s="35" t="inlineStr">
+        <is>
+          <t>CPL EMASON SAUTET</t>
+        </is>
+      </c>
+      <c r="M25" s="34" t="inlineStr">
         <is>
           <t>LEGAL</t>
         </is>
       </c>
-      <c r="N25" s="34" t="inlineStr"/>
+      <c r="N25" s="35" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>